<commit_message>
updating some data files
</commit_message>
<xml_diff>
--- a/data/ADMIN Ledger 2024-5.xlsx
+++ b/data/ADMIN Ledger 2024-5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dannelson/Desktop/we-serve/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271C2876-94BA-7642-9C32-04CB8E094756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3E090F-3AE1-734C-BA70-11751D3AE31F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="960" windowWidth="27640" windowHeight="16940" xr2:uid="{FE5CA08C-29D2-4840-9FF4-E51BBBAA1191}"/>
+    <workbookView xWindow="0" yWindow="940" windowWidth="27640" windowHeight="16940" xr2:uid="{FE5CA08C-29D2-4840-9FF4-E51BBBAA1191}"/>
   </bookViews>
   <sheets>
     <sheet name="Ledger 2024-5" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="77">
   <si>
     <t>ID</t>
   </si>
@@ -185,12 +185,6 @@
     <t>24/10/31</t>
   </si>
   <si>
-    <t>24/11/4</t>
-  </si>
-  <si>
-    <t>Liberty Mutual Ins</t>
-  </si>
-  <si>
     <t>24/11/18</t>
   </si>
   <si>
@@ -266,9 +260,6 @@
     <t>25/3/20</t>
   </si>
   <si>
-    <t>Sue Schmoker</t>
-  </si>
-  <si>
     <t>Anita Wilkie</t>
   </si>
   <si>
@@ -276,6 +267,9 @@
   </si>
   <si>
     <t>25/4/18</t>
+  </si>
+  <si>
+    <t>Sue Schmoker, flowers for Wilkies</t>
   </si>
 </sst>
 </file>
@@ -834,11 +828,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A645121C-3F67-D346-9F8D-BAE6E6139A06}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" style="2"/>
     <col min="5" max="5" width="11.1640625" style="4" customWidth="1"/>
@@ -895,6 +889,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
+        <f>A2+1</f>
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -920,6 +915,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
+        <f t="shared" ref="A4:A58" si="0">A3+1</f>
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -944,6 +940,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" t="s">
@@ -968,7 +965,8 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>6</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -992,7 +990,8 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>7</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
@@ -1016,7 +1015,8 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -1040,7 +1040,8 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>9</v>
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
@@ -1064,7 +1065,8 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
@@ -1088,7 +1090,8 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>11</v>
+        <f t="shared" si="0"/>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
@@ -1112,7 +1115,8 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>12</v>
+        <f t="shared" si="0"/>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
@@ -1136,7 +1140,8 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>13</v>
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
@@ -1161,7 +1166,8 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>14</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>23</v>
@@ -1185,7 +1191,8 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>24</v>
@@ -1209,7 +1216,8 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>16</v>
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>25</v>
@@ -1233,7 +1241,8 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>17</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>27</v>
@@ -1257,7 +1266,8 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>18</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>28</v>
@@ -1281,7 +1291,8 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>28</v>
@@ -1305,7 +1316,8 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
@@ -1329,7 +1341,8 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>21</v>
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>32</v>
@@ -1353,7 +1366,8 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>34</v>
@@ -1377,7 +1391,8 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>35</v>
@@ -1401,7 +1416,8 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>24</v>
+        <f t="shared" si="0"/>
+        <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -1425,7 +1441,8 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>38</v>
@@ -1449,7 +1466,8 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
         <v>39</v>
@@ -1473,7 +1491,8 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
@@ -1497,7 +1516,8 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>41</v>
@@ -1521,7 +1541,8 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>42</v>
@@ -1545,7 +1566,8 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
         <v>43</v>
@@ -1569,7 +1591,8 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
-        <v>31</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
         <v>44</v>
@@ -1593,7 +1616,8 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
         <v>47</v>
@@ -1617,7 +1641,8 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
         <v>48</v>
@@ -1625,11 +1650,11 @@
       <c r="C33" t="s">
         <v>49</v>
       </c>
-      <c r="D33" s="2">
-        <v>3146</v>
+      <c r="D33" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E33" s="4">
-        <v>425</v>
+        <v>2500</v>
       </c>
       <c r="F33" s="2">
         <v>110</v>
@@ -1641,115 +1666,120 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C34" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E34" s="4">
-        <v>2500</v>
+        <v>81</v>
       </c>
       <c r="F34" s="2">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="G34" t="str">
         <f>VLOOKUP(F34,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Donations</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
         <v>50</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="E35" s="4">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="F35" s="2">
-        <v>150</v>
+        <v>110</v>
       </c>
       <c r="G35" t="str">
         <f>VLOOKUP(F35,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Donations</v>
+        <v>Misc.Income &amp; Expenses</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36">
-        <v>36</v>
+        <f t="shared" si="0"/>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C36" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="E36" s="4">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F36" s="2">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="G36" t="str">
         <f>VLOOKUP(F36,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37">
-        <v>37</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C37" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E37" s="4">
-        <v>16</v>
+        <v>150</v>
       </c>
       <c r="F37" s="2">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G37" t="str">
         <f>VLOOKUP(F37,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Misc.Income &amp; Expenses</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>38</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>55</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>10</v>
+        <v>54</v>
+      </c>
+      <c r="D38" s="2">
+        <v>3147</v>
       </c>
       <c r="E38" s="4">
-        <v>150</v>
+        <v>9.52</v>
       </c>
       <c r="F38" s="2">
         <v>110</v>
@@ -1761,58 +1791,61 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39">
-        <v>39</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C39" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" s="2">
-        <v>3147</v>
+        <v>22</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E39" s="4">
-        <v>9.52</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F39" s="2">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G39" t="str">
         <f>VLOOKUP(F39,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Interest on Bank Account</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>40</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C40" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E40" s="4">
-        <v>7.0000000000000007E-2</v>
+        <v>23</v>
       </c>
       <c r="F40" s="2">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="G40" t="str">
         <f>VLOOKUP(F40,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Interest on Bank Account</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>41</v>
+        <f t="shared" si="0"/>
+        <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C41" t="s">
         <v>37</v>
@@ -1821,7 +1854,7 @@
         <v>10</v>
       </c>
       <c r="E41" s="4">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F41" s="2">
         <v>140</v>
@@ -1833,151 +1866,158 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42">
-        <v>42</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C42" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E42" s="4">
-        <v>16</v>
+        <v>0.09</v>
       </c>
       <c r="F42" s="2">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="G42" t="str">
         <f>VLOOKUP(F42,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Interest on Bank Account</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43">
-        <v>43</v>
+        <f t="shared" si="0"/>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C43" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E43" s="4">
-        <v>0.09</v>
+        <v>12.5</v>
       </c>
       <c r="F43" s="2">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="G43" t="str">
         <f>VLOOKUP(F43,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Interest on Bank Account</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44">
-        <v>44</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C44" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E44" s="4">
-        <v>12.5</v>
+        <v>50</v>
       </c>
       <c r="F44" s="2">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="G44" t="str">
         <f>VLOOKUP(F44,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Donations</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45">
-        <v>45</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
         <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>10</v>
+        <v>60</v>
+      </c>
+      <c r="D45" s="2">
+        <v>3027</v>
       </c>
       <c r="E45" s="4">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="F45" s="2">
-        <v>150</v>
+        <v>110</v>
       </c>
       <c r="G45" t="str">
         <f>VLOOKUP(F45,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Donations</v>
+        <v>Misc.Income &amp; Expenses</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46">
-        <v>46</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>62</v>
-      </c>
-      <c r="D46" s="2">
-        <v>3027</v>
+        <v>37</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E46" s="4">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="F46" s="2">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="G46" t="str">
         <f>VLOOKUP(F46,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47">
-        <v>47</v>
+        <f t="shared" si="0"/>
+        <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>63</v>
+      </c>
+      <c r="C47" t="s">
         <v>64</v>
       </c>
-      <c r="C47" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>10</v>
+      <c r="D47" s="2">
+        <v>3030</v>
       </c>
       <c r="E47" s="4">
-        <v>20</v>
+        <v>19.010000000000002</v>
       </c>
       <c r="F47" s="2">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="G47" t="str">
         <f>VLOOKUP(F47,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Guest Dinners</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48">
-        <v>48</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
       <c r="B48" t="s">
         <v>65</v>
@@ -1986,241 +2026,251 @@
         <v>66</v>
       </c>
       <c r="D48" s="2">
-        <v>3030</v>
+        <v>3148</v>
       </c>
       <c r="E48" s="4">
-        <v>19.010000000000002</v>
+        <v>1265.51</v>
       </c>
       <c r="F48" s="2">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G48" t="str">
         <f>VLOOKUP(F48,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Guest Dinners</v>
+        <v xml:space="preserve">   MD19 Capita Dues - Expense $26.60</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49">
-        <v>49</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
       <c r="B49" t="s">
         <v>67</v>
       </c>
       <c r="C49" t="s">
-        <v>68</v>
-      </c>
-      <c r="D49" s="2">
-        <v>3148</v>
+        <v>22</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E49" s="4">
-        <v>1265.51</v>
+        <v>0.09</v>
       </c>
       <c r="F49" s="2">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G49" t="str">
         <f>VLOOKUP(F49,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v xml:space="preserve">   MD19 Capita Dues - Expense $26.60</v>
+        <v>Interest on Bank Account</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50">
-        <v>50</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C50" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E50" s="4">
-        <v>0.09</v>
+        <v>18</v>
       </c>
       <c r="F50" s="2">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="G50" t="str">
         <f>VLOOKUP(F50,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Interest on Bank Account</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51">
-        <v>51</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C51" t="s">
-        <v>37</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>10</v>
+        <v>29</v>
+      </c>
+      <c r="D51" s="2">
+        <v>3149</v>
       </c>
       <c r="E51" s="4">
-        <v>18</v>
+        <v>684</v>
       </c>
       <c r="F51" s="2">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="G51" t="str">
         <f>VLOOKUP(F51,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v xml:space="preserve">   LCI Capita Dues -  Expense @ $48.00</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52">
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C52" t="s">
-        <v>29</v>
-      </c>
-      <c r="D52" s="2">
-        <v>3149</v>
+        <v>37</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E52" s="4">
-        <v>684</v>
+        <v>13</v>
       </c>
       <c r="F52" s="2">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="G52" t="str">
         <f>VLOOKUP(F52,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v xml:space="preserve">   LCI Capita Dues -  Expense @ $48.00</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53">
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>70</v>
+      </c>
+      <c r="C53" t="s">
         <v>71</v>
       </c>
-      <c r="C53" t="s">
-        <v>37</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>10</v>
+      <c r="D53" s="2">
+        <v>3029</v>
       </c>
       <c r="E53" s="4">
-        <v>13</v>
+        <v>210</v>
       </c>
       <c r="F53" s="2">
-        <v>140</v>
+        <v>10</v>
       </c>
       <c r="G53" t="str">
         <f>VLOOKUP(F53,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Bulletin,Postage, Box Rental</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54">
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
       <c r="B54" t="s">
         <v>72</v>
       </c>
       <c r="C54" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D54" s="2">
-        <v>3029</v>
+        <v>3031</v>
       </c>
       <c r="E54" s="4">
-        <v>210</v>
+        <v>29.31</v>
       </c>
       <c r="F54" s="2">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="G54" t="str">
         <f>VLOOKUP(F54,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Bulletin,Postage, Box Rental</v>
+        <v>Misc.Income &amp; Expenses</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55">
-        <v>53</v>
+        <f t="shared" si="0"/>
+        <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C55" t="s">
-        <v>75</v>
-      </c>
-      <c r="D55" s="2">
-        <v>3031</v>
+        <v>37</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E55" s="4">
-        <v>29.31</v>
+        <v>9</v>
       </c>
       <c r="F55" s="2">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="G55" t="str">
         <f>VLOOKUP(F55,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C56" t="s">
-        <v>37</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>10</v>
+        <v>73</v>
+      </c>
+      <c r="D56" s="2">
+        <v>3032</v>
       </c>
       <c r="E56" s="4">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="F56" s="2">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G56" t="str">
         <f>VLOOKUP(F56,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
+        <v>Misc.Income &amp; Expenses</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57">
-        <v>55</v>
+        <f t="shared" si="0"/>
+        <v>56</v>
       </c>
       <c r="B57" t="s">
         <v>74</v>
       </c>
       <c r="C57" t="s">
-        <v>76</v>
-      </c>
-      <c r="D57" s="2">
-        <v>3032</v>
+        <v>37</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E57" s="4">
-        <v>130</v>
+        <v>23</v>
       </c>
       <c r="F57" s="2">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="G57" t="str">
         <f>VLOOKUP(F57,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Misc.Income &amp; Expenses</v>
+        <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58">
-        <v>55</v>
+        <f t="shared" si="0"/>
+        <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C58" t="s">
         <v>37</v>
@@ -2229,37 +2279,13 @@
         <v>10</v>
       </c>
       <c r="E58" s="4">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F58" s="2">
         <v>140</v>
       </c>
       <c r="G58" t="str">
         <f>VLOOKUP(F58,[1]budgets!$A$4:$B$20,2,FALSE)</f>
-        <v>Tail Twisting/Happy Bucks</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A59">
-        <v>56</v>
-      </c>
-      <c r="B59" t="s">
-        <v>78</v>
-      </c>
-      <c r="C59" t="s">
-        <v>37</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" s="4">
-        <v>10</v>
-      </c>
-      <c r="F59" s="2">
-        <v>140</v>
-      </c>
-      <c r="G59" t="str">
-        <f>VLOOKUP(F59,[1]budgets!$A$4:$B$20,2,FALSE)</f>
         <v>Tail Twisting/Happy Bucks</v>
       </c>
     </row>

</xml_diff>